<commit_message>
Auto backup 2026-07-02 03:35:01
</commit_message>
<xml_diff>
--- a/SwissTechSaqib/Swiss Tech Files 2025/Profit Reports/profit report.xlsx
+++ b/SwissTechSaqib/Swiss Tech Files 2025/Profit Reports/profit report.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\dell5300\Documents\Swiss Tech Files 2025\Profit Reports\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\SwissTechSaqib\Swiss Tech Files 2025\Profit Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F553B5C5-824B-414F-99A7-FC3C3DDE5806}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5177570A-BA1A-404C-8D58-84200F20C6BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="2" xr2:uid="{C511F85B-2D97-4B40-9A5D-0F8673C41C5B}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C511F85B-2D97-4B40-9A5D-0F8673C41C5B}"/>
   </bookViews>
   <sheets>
     <sheet name="Company Worth" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1242" uniqueCount="363">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1259" uniqueCount="365">
   <si>
     <t>Total Stock Worth</t>
   </si>
@@ -1520,6 +1520,12 @@
       </rPr>
       <t xml:space="preserve"> 11,598.54</t>
     </r>
+  </si>
+  <si>
+    <t>Income Statement For June-2026</t>
+  </si>
+  <si>
+    <t>Khi Carry &amp; Shop Exp</t>
   </si>
 </sst>
 </file>
@@ -1863,10 +1869,10 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -8850,11 +8856,6 @@
     </row>
   </sheetData>
   <mergeCells count="13">
-    <mergeCell ref="E569:F569"/>
-    <mergeCell ref="H510:I510"/>
-    <mergeCell ref="E391:F391"/>
-    <mergeCell ref="E283:F283"/>
-    <mergeCell ref="E335:F335"/>
     <mergeCell ref="E234:F234"/>
     <mergeCell ref="E508:F508"/>
     <mergeCell ref="E448:F448"/>
@@ -8863,6 +8864,11 @@
     <mergeCell ref="E94:F94"/>
     <mergeCell ref="E140:F140"/>
     <mergeCell ref="E188:F188"/>
+    <mergeCell ref="E569:F569"/>
+    <mergeCell ref="H510:I510"/>
+    <mergeCell ref="E391:F391"/>
+    <mergeCell ref="E283:F283"/>
+    <mergeCell ref="E335:F335"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -8872,7 +8878,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{16B3874F-7CF8-4B81-A570-F17A1D413ED0}">
   <sheetPr codeName="Sheet2"/>
-  <dimension ref="B2:I538"/>
+  <dimension ref="B2:I580"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11" customWidth="1"/>
@@ -8885,24 +8891,24 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B2" s="62" t="s">
+      <c r="B2" s="63" t="s">
         <v>196</v>
       </c>
-      <c r="C2" s="62"/>
-      <c r="H2" s="62" t="s">
+      <c r="C2" s="63"/>
+      <c r="H2" s="63" t="s">
         <v>197</v>
       </c>
-      <c r="I2" s="62"/>
+      <c r="I2" s="63"/>
     </row>
     <row r="4" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B4" s="63" t="s">
+      <c r="B4" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C4" s="63"/>
-      <c r="H4" s="63" t="s">
+      <c r="C4" s="62"/>
+      <c r="H4" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="I4" s="63"/>
+      <c r="I4" s="62"/>
     </row>
     <row r="5" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B5" s="18" t="s">
@@ -8955,14 +8961,14 @@
       <c r="I8" s="20"/>
     </row>
     <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B9" s="63" t="s">
+      <c r="B9" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C9" s="63"/>
-      <c r="H9" s="63" t="s">
+      <c r="C9" s="62"/>
+      <c r="H9" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="I9" s="63"/>
+      <c r="I9" s="62"/>
     </row>
     <row r="10" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B10" s="18" t="s">
@@ -9007,14 +9013,14 @@
       <c r="I13" s="20"/>
     </row>
     <row r="14" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B14" s="63" t="s">
+      <c r="B14" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C14" s="63"/>
-      <c r="H14" s="63" t="s">
+      <c r="C14" s="62"/>
+      <c r="H14" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="I14" s="63"/>
+      <c r="I14" s="62"/>
     </row>
     <row r="15" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B15" s="18" t="s">
@@ -9135,10 +9141,10 @@
       </c>
     </row>
     <row r="29" spans="2:9" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B29" s="62" t="s">
+      <c r="B29" s="63" t="s">
         <v>213</v>
       </c>
-      <c r="C29" s="62"/>
+      <c r="C29" s="63"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H30" t="s">
@@ -9146,10 +9152,10 @@
       </c>
     </row>
     <row r="32" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B32" s="63" t="s">
+      <c r="B32" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C32" s="63"/>
+      <c r="C32" s="62"/>
     </row>
     <row r="33" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B33" s="18" t="s">
@@ -9186,10 +9192,10 @@
       <c r="C36" s="20"/>
     </row>
     <row r="37" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B37" s="63" t="s">
+      <c r="B37" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C37" s="63"/>
+      <c r="C37" s="62"/>
     </row>
     <row r="38" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B38" s="18" t="s">
@@ -9218,10 +9224,10 @@
       <c r="C41" s="20"/>
     </row>
     <row r="42" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B42" s="63" t="s">
+      <c r="B42" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C42" s="63"/>
+      <c r="C42" s="62"/>
     </row>
     <row r="43" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B43" s="18" t="s">
@@ -9296,16 +9302,16 @@
       </c>
     </row>
     <row r="58" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B58" s="62" t="s">
+      <c r="B58" s="63" t="s">
         <v>215</v>
       </c>
-      <c r="C58" s="62"/>
+      <c r="C58" s="63"/>
     </row>
     <row r="61" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B61" s="63" t="s">
+      <c r="B61" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C61" s="63"/>
+      <c r="C61" s="62"/>
     </row>
     <row r="62" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B62" s="18" t="s">
@@ -9337,10 +9343,10 @@
       <c r="C65" s="20"/>
     </row>
     <row r="66" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B66" s="63" t="s">
+      <c r="B66" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C66" s="63"/>
+      <c r="C66" s="62"/>
     </row>
     <row r="67" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B67" s="18" t="s">
@@ -9368,10 +9374,10 @@
       <c r="C70" s="20"/>
     </row>
     <row r="71" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B71" s="63" t="s">
+      <c r="B71" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C71" s="63"/>
+      <c r="C71" s="62"/>
     </row>
     <row r="72" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B72" s="18" t="s">
@@ -9456,16 +9462,16 @@
       </c>
     </row>
     <row r="89" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B89" s="62" t="s">
+      <c r="B89" s="63" t="s">
         <v>218</v>
       </c>
-      <c r="C89" s="62"/>
+      <c r="C89" s="63"/>
     </row>
     <row r="92" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B92" s="63" t="s">
+      <c r="B92" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C92" s="63"/>
+      <c r="C92" s="62"/>
     </row>
     <row r="93" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B93" s="18" t="s">
@@ -9497,10 +9503,10 @@
       <c r="C96" s="20"/>
     </row>
     <row r="97" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B97" s="63" t="s">
+      <c r="B97" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C97" s="63"/>
+      <c r="C97" s="62"/>
     </row>
     <row r="98" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B98" s="18" t="s">
@@ -9528,10 +9534,10 @@
       <c r="C101" s="20"/>
     </row>
     <row r="102" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B102" s="63" t="s">
+      <c r="B102" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C102" s="63"/>
+      <c r="C102" s="62"/>
     </row>
     <row r="103" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B103" s="18" t="s">
@@ -9612,16 +9618,16 @@
       </c>
     </row>
     <row r="118" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B118" s="62" t="s">
+      <c r="B118" s="63" t="s">
         <v>219</v>
       </c>
-      <c r="C118" s="62"/>
+      <c r="C118" s="63"/>
     </row>
     <row r="121" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B121" s="63" t="s">
+      <c r="B121" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C121" s="63"/>
+      <c r="C121" s="62"/>
     </row>
     <row r="122" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B122" s="18" t="s">
@@ -9653,10 +9659,10 @@
       <c r="C125" s="20"/>
     </row>
     <row r="126" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B126" s="63" t="s">
+      <c r="B126" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C126" s="63"/>
+      <c r="C126" s="62"/>
     </row>
     <row r="127" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B127" s="18" t="s">
@@ -9684,10 +9690,10 @@
       <c r="C130" s="20"/>
     </row>
     <row r="131" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B131" s="63" t="s">
+      <c r="B131" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C131" s="63"/>
+      <c r="C131" s="62"/>
     </row>
     <row r="132" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B132" s="18" t="s">
@@ -9772,16 +9778,16 @@
       </c>
     </row>
     <row r="151" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B151" s="62" t="s">
+      <c r="B151" s="63" t="s">
         <v>220</v>
       </c>
-      <c r="C151" s="62"/>
+      <c r="C151" s="63"/>
     </row>
     <row r="154" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B154" s="63" t="s">
+      <c r="B154" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C154" s="63"/>
+      <c r="C154" s="62"/>
     </row>
     <row r="155" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B155" s="18" t="s">
@@ -9813,10 +9819,10 @@
       <c r="C158" s="20"/>
     </row>
     <row r="159" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B159" s="63" t="s">
+      <c r="B159" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C159" s="63"/>
+      <c r="C159" s="62"/>
     </row>
     <row r="160" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B160" s="18" t="s">
@@ -9844,10 +9850,10 @@
       <c r="C163" s="20"/>
     </row>
     <row r="164" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B164" s="63" t="s">
+      <c r="B164" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C164" s="63"/>
+      <c r="C164" s="62"/>
     </row>
     <row r="165" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B165" s="18" t="s">
@@ -9952,16 +9958,16 @@
       </c>
     </row>
     <row r="185" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B185" s="62" t="s">
+      <c r="B185" s="63" t="s">
         <v>224</v>
       </c>
-      <c r="C185" s="62"/>
+      <c r="C185" s="63"/>
     </row>
     <row r="188" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B188" s="63" t="s">
+      <c r="B188" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C188" s="63"/>
+      <c r="C188" s="62"/>
     </row>
     <row r="189" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B189" s="18" t="s">
@@ -9993,10 +9999,10 @@
       <c r="C192" s="20"/>
     </row>
     <row r="193" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B193" s="63" t="s">
+      <c r="B193" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C193" s="63"/>
+      <c r="C193" s="62"/>
     </row>
     <row r="194" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B194" s="18" t="s">
@@ -10024,10 +10030,10 @@
       <c r="C197" s="20"/>
     </row>
     <row r="198" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B198" s="63" t="s">
+      <c r="B198" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C198" s="63"/>
+      <c r="C198" s="62"/>
     </row>
     <row r="199" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B199" s="18" t="s">
@@ -10128,16 +10134,16 @@
       </c>
     </row>
     <row r="215" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B215" s="62" t="s">
+      <c r="B215" s="63" t="s">
         <v>225</v>
       </c>
-      <c r="C215" s="62"/>
+      <c r="C215" s="63"/>
     </row>
     <row r="218" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B218" s="63" t="s">
+      <c r="B218" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C218" s="63"/>
+      <c r="C218" s="62"/>
     </row>
     <row r="219" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B219" s="18" t="s">
@@ -10169,10 +10175,10 @@
       <c r="C222" s="20"/>
     </row>
     <row r="223" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B223" s="63" t="s">
+      <c r="B223" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C223" s="63"/>
+      <c r="C223" s="62"/>
     </row>
     <row r="224" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B224" s="18" t="s">
@@ -10200,10 +10206,10 @@
       <c r="C227" s="20"/>
     </row>
     <row r="228" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B228" s="63" t="s">
+      <c r="B228" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C228" s="63"/>
+      <c r="C228" s="62"/>
     </row>
     <row r="229" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B229" s="18" t="s">
@@ -10310,16 +10316,16 @@
       </c>
     </row>
     <row r="246" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B246" s="62" t="s">
+      <c r="B246" s="63" t="s">
         <v>228</v>
       </c>
-      <c r="C246" s="62"/>
+      <c r="C246" s="63"/>
     </row>
     <row r="249" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B249" s="63" t="s">
+      <c r="B249" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C249" s="63"/>
+      <c r="C249" s="62"/>
     </row>
     <row r="250" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B250" s="18" t="s">
@@ -10351,10 +10357,10 @@
       <c r="C253" s="20"/>
     </row>
     <row r="254" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B254" s="63" t="s">
+      <c r="B254" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C254" s="63"/>
+      <c r="C254" s="62"/>
     </row>
     <row r="255" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B255" s="18" t="s">
@@ -10382,10 +10388,10 @@
       <c r="C258" s="20"/>
     </row>
     <row r="259" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B259" s="63" t="s">
+      <c r="B259" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C259" s="63"/>
+      <c r="C259" s="62"/>
     </row>
     <row r="260" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B260" s="18" t="s">
@@ -10508,16 +10514,16 @@
       </c>
     </row>
     <row r="283" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B283" s="62" t="s">
+      <c r="B283" s="63" t="s">
         <v>231</v>
       </c>
-      <c r="C283" s="62"/>
+      <c r="C283" s="63"/>
     </row>
     <row r="286" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B286" s="63" t="s">
+      <c r="B286" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C286" s="63"/>
+      <c r="C286" s="62"/>
     </row>
     <row r="287" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B287" s="18" t="s">
@@ -10549,10 +10555,10 @@
       <c r="C290" s="20"/>
     </row>
     <row r="291" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B291" s="63" t="s">
+      <c r="B291" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C291" s="63"/>
+      <c r="C291" s="62"/>
     </row>
     <row r="292" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B292" s="18" t="s">
@@ -10580,10 +10586,10 @@
       <c r="C295" s="20"/>
     </row>
     <row r="296" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B296" s="63" t="s">
+      <c r="B296" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C296" s="63"/>
+      <c r="C296" s="62"/>
     </row>
     <row r="297" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B297" s="18" t="s">
@@ -10698,16 +10704,16 @@
       </c>
     </row>
     <row r="323" spans="2:8" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B323" s="62" t="s">
+      <c r="B323" s="63" t="s">
         <v>232</v>
       </c>
-      <c r="C323" s="62"/>
+      <c r="C323" s="63"/>
     </row>
     <row r="326" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B326" s="63" t="s">
+      <c r="B326" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C326" s="63"/>
+      <c r="C326" s="62"/>
     </row>
     <row r="327" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B327" s="18" t="s">
@@ -10742,10 +10748,10 @@
       <c r="C330" s="20"/>
     </row>
     <row r="331" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B331" s="63" t="s">
+      <c r="B331" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C331" s="63"/>
+      <c r="C331" s="62"/>
     </row>
     <row r="332" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B332" s="18" t="s">
@@ -10773,10 +10779,10 @@
       <c r="C335" s="20"/>
     </row>
     <row r="336" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B336" s="63" t="s">
+      <c r="B336" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C336" s="63"/>
+      <c r="C336" s="62"/>
     </row>
     <row r="337" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B337" s="18" t="s">
@@ -10869,16 +10875,16 @@
       </c>
     </row>
     <row r="359" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B359" s="62" t="s">
+      <c r="B359" s="63" t="s">
         <v>259</v>
       </c>
-      <c r="C359" s="62"/>
+      <c r="C359" s="63"/>
     </row>
     <row r="362" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B362" s="63" t="s">
+      <c r="B362" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C362" s="63"/>
+      <c r="C362" s="62"/>
     </row>
     <row r="363" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B363" s="18" t="s">
@@ -10910,10 +10916,10 @@
       <c r="C366" s="20"/>
     </row>
     <row r="367" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B367" s="63" t="s">
+      <c r="B367" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C367" s="63"/>
+      <c r="C367" s="62"/>
     </row>
     <row r="368" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B368" s="18" t="s">
@@ -10941,10 +10947,10 @@
       <c r="C371" s="20"/>
     </row>
     <row r="372" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B372" s="63" t="s">
+      <c r="B372" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C372" s="63"/>
+      <c r="C372" s="62"/>
     </row>
     <row r="373" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B373" s="18" t="s">
@@ -11041,16 +11047,16 @@
       </c>
     </row>
     <row r="395" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B395" s="62" t="s">
+      <c r="B395" s="63" t="s">
         <v>302</v>
       </c>
-      <c r="C395" s="62"/>
+      <c r="C395" s="63"/>
     </row>
     <row r="398" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B398" s="63" t="s">
+      <c r="B398" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C398" s="63"/>
+      <c r="C398" s="62"/>
     </row>
     <row r="399" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B399" s="18" t="s">
@@ -11082,10 +11088,10 @@
       <c r="C402" s="20"/>
     </row>
     <row r="403" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B403" s="63" t="s">
+      <c r="B403" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C403" s="63"/>
+      <c r="C403" s="62"/>
     </row>
     <row r="404" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B404" s="18" t="s">
@@ -11113,10 +11119,10 @@
       <c r="C407" s="20"/>
     </row>
     <row r="408" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B408" s="63" t="s">
+      <c r="B408" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C408" s="63"/>
+      <c r="C408" s="62"/>
     </row>
     <row r="409" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B409" s="18" t="s">
@@ -11213,16 +11219,16 @@
       </c>
     </row>
     <row r="432" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B432" s="62" t="s">
+      <c r="B432" s="63" t="s">
         <v>314</v>
       </c>
-      <c r="C432" s="62"/>
+      <c r="C432" s="63"/>
     </row>
     <row r="435" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B435" s="63" t="s">
+      <c r="B435" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C435" s="63"/>
+      <c r="C435" s="62"/>
     </row>
     <row r="436" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B436" s="18" t="s">
@@ -11254,10 +11260,10 @@
       <c r="C439" s="20"/>
     </row>
     <row r="440" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B440" s="63" t="s">
+      <c r="B440" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C440" s="63"/>
+      <c r="C440" s="62"/>
     </row>
     <row r="441" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B441" s="18" t="s">
@@ -11285,10 +11291,10 @@
       <c r="C444" s="20"/>
     </row>
     <row r="445" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B445" s="63" t="s">
+      <c r="B445" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C445" s="63"/>
+      <c r="C445" s="62"/>
     </row>
     <row r="446" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B446" s="18" t="s">
@@ -11385,16 +11391,16 @@
       </c>
     </row>
     <row r="470" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B470" s="62" t="s">
+      <c r="B470" s="63" t="s">
         <v>321</v>
       </c>
-      <c r="C470" s="62"/>
+      <c r="C470" s="63"/>
     </row>
     <row r="473" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B473" s="63" t="s">
+      <c r="B473" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C473" s="63"/>
+      <c r="C473" s="62"/>
     </row>
     <row r="474" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B474" s="18" t="s">
@@ -11426,10 +11432,10 @@
       <c r="C477" s="20"/>
     </row>
     <row r="478" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B478" s="63" t="s">
+      <c r="B478" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C478" s="63"/>
+      <c r="C478" s="62"/>
     </row>
     <row r="479" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B479" s="18" t="s">
@@ -11457,10 +11463,10 @@
       <c r="C482" s="20"/>
     </row>
     <row r="483" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B483" s="63" t="s">
+      <c r="B483" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C483" s="63"/>
+      <c r="C483" s="62"/>
     </row>
     <row r="484" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B484" s="18" t="s">
@@ -11557,16 +11563,16 @@
       </c>
     </row>
     <row r="510" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B510" s="62" t="s">
+      <c r="B510" s="63" t="s">
         <v>328</v>
       </c>
-      <c r="C510" s="62"/>
+      <c r="C510" s="63"/>
     </row>
     <row r="513" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B513" s="63" t="s">
+      <c r="B513" s="62" t="s">
         <v>198</v>
       </c>
-      <c r="C513" s="63"/>
+      <c r="C513" s="62"/>
     </row>
     <row r="514" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B514" s="18" t="s">
@@ -11598,10 +11604,10 @@
       <c r="C517" s="20"/>
     </row>
     <row r="518" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B518" s="63" t="s">
+      <c r="B518" s="62" t="s">
         <v>202</v>
       </c>
-      <c r="C518" s="63"/>
+      <c r="C518" s="62"/>
     </row>
     <row r="519" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B519" s="18" t="s">
@@ -11629,10 +11635,10 @@
       <c r="C522" s="20"/>
     </row>
     <row r="523" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B523" s="63" t="s">
+      <c r="B523" s="62" t="s">
         <v>205</v>
       </c>
-      <c r="C523" s="63"/>
+      <c r="C523" s="62"/>
     </row>
     <row r="524" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B524" s="18" t="s">
@@ -11728,17 +11734,223 @@
         <v>342987.69463127549</v>
       </c>
     </row>
+    <row r="552" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="B552" s="63" t="s">
+        <v>363</v>
+      </c>
+      <c r="C552" s="63"/>
+    </row>
+    <row r="555" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B555" s="62" t="s">
+        <v>198</v>
+      </c>
+      <c r="C555" s="62"/>
+    </row>
+    <row r="556" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B556" s="18" t="s">
+        <v>199</v>
+      </c>
+      <c r="C556" s="19">
+        <v>1915429.34</v>
+      </c>
+    </row>
+    <row r="557" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B557" s="18" t="s">
+        <v>200</v>
+      </c>
+      <c r="C557" s="19">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="558" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B558" s="18" t="s">
+        <v>201</v>
+      </c>
+      <c r="C558" s="19">
+        <f>C556-C557</f>
+        <v>1915429.34</v>
+      </c>
+    </row>
+    <row r="559" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B559" s="20"/>
+      <c r="C559" s="20"/>
+    </row>
+    <row r="560" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B560" s="62" t="s">
+        <v>202</v>
+      </c>
+      <c r="C560" s="62"/>
+    </row>
+    <row r="561" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B561" s="18" t="s">
+        <v>203</v>
+      </c>
+      <c r="C561" s="19">
+        <v>1545654.22</v>
+      </c>
+    </row>
+    <row r="562" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B562" s="21"/>
+      <c r="C562" s="20"/>
+    </row>
+    <row r="563" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B563" s="18" t="s">
+        <v>204</v>
+      </c>
+      <c r="C563" s="19">
+        <f>C558-C561</f>
+        <v>369775.12000000011</v>
+      </c>
+    </row>
+    <row r="564" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B564" s="20"/>
+      <c r="C564" s="20"/>
+    </row>
+    <row r="565" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B565" s="62" t="s">
+        <v>205</v>
+      </c>
+      <c r="C565" s="62"/>
+    </row>
+    <row r="566" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B566" s="18" t="s">
+        <v>206</v>
+      </c>
+      <c r="C566" s="19">
+        <v>109079.26000000001</v>
+      </c>
+    </row>
+    <row r="567" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B567" s="18"/>
+      <c r="C567" s="19"/>
+    </row>
+    <row r="568" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B568" s="18"/>
+      <c r="C568" s="19"/>
+    </row>
+    <row r="569" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B569" s="18"/>
+      <c r="C569" s="19"/>
+    </row>
+    <row r="570" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B570" s="18"/>
+      <c r="C570" s="19"/>
+    </row>
+    <row r="571" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B571" s="18"/>
+      <c r="C571" s="19"/>
+    </row>
+    <row r="572" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B572" s="18" t="s">
+        <v>260</v>
+      </c>
+      <c r="C572" s="19"/>
+    </row>
+    <row r="573" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B573" s="18" t="s">
+        <v>221</v>
+      </c>
+      <c r="C573" s="19">
+        <v>29138.079999999998</v>
+      </c>
+    </row>
+    <row r="574" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B574" s="18" t="s">
+        <v>222</v>
+      </c>
+      <c r="C574" s="19">
+        <v>45245.64</v>
+      </c>
+    </row>
+    <row r="575" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B575" s="18" t="s">
+        <v>227</v>
+      </c>
+      <c r="C575" s="19"/>
+    </row>
+    <row r="576" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B576" s="18" t="s">
+        <v>364</v>
+      </c>
+      <c r="C576" s="19">
+        <v>9846.7999999999993</v>
+      </c>
+    </row>
+    <row r="577" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B577" s="20"/>
+      <c r="C577" s="20"/>
+    </row>
+    <row r="578" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B578" s="18" t="s">
+        <v>211</v>
+      </c>
+      <c r="C578" s="19">
+        <f>SUM(C566:C577)</f>
+        <v>193309.77999999997</v>
+      </c>
+    </row>
+    <row r="579" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="B579" s="21"/>
+      <c r="C579" s="24"/>
+    </row>
+    <row r="580" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
+      <c r="B580" s="22" t="s">
+        <v>212</v>
+      </c>
+      <c r="C580" s="23">
+        <f>C563-C578</f>
+        <v>176465.34000000014</v>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="68">
-    <mergeCell ref="B102:C102"/>
-    <mergeCell ref="B118:C118"/>
-    <mergeCell ref="B121:C121"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="H9:I9"/>
+  <mergeCells count="72">
+    <mergeCell ref="B552:C552"/>
+    <mergeCell ref="B555:C555"/>
+    <mergeCell ref="B560:C560"/>
+    <mergeCell ref="B565:C565"/>
+    <mergeCell ref="B510:C510"/>
+    <mergeCell ref="B513:C513"/>
+    <mergeCell ref="B518:C518"/>
+    <mergeCell ref="B523:C523"/>
+    <mergeCell ref="B470:C470"/>
+    <mergeCell ref="B473:C473"/>
+    <mergeCell ref="B478:C478"/>
+    <mergeCell ref="B483:C483"/>
+    <mergeCell ref="B432:C432"/>
+    <mergeCell ref="B435:C435"/>
+    <mergeCell ref="B440:C440"/>
+    <mergeCell ref="B445:C445"/>
+    <mergeCell ref="B395:C395"/>
+    <mergeCell ref="B398:C398"/>
+    <mergeCell ref="B403:C403"/>
+    <mergeCell ref="B408:C408"/>
+    <mergeCell ref="B367:C367"/>
+    <mergeCell ref="B372:C372"/>
+    <mergeCell ref="B336:C336"/>
+    <mergeCell ref="B254:C254"/>
+    <mergeCell ref="B259:C259"/>
+    <mergeCell ref="B283:C283"/>
+    <mergeCell ref="B359:C359"/>
+    <mergeCell ref="B291:C291"/>
+    <mergeCell ref="B296:C296"/>
+    <mergeCell ref="B323:C323"/>
+    <mergeCell ref="B326:C326"/>
+    <mergeCell ref="B331:C331"/>
+    <mergeCell ref="B362:C362"/>
+    <mergeCell ref="B286:C286"/>
+    <mergeCell ref="B126:C126"/>
+    <mergeCell ref="B228:C228"/>
+    <mergeCell ref="B151:C151"/>
+    <mergeCell ref="B154:C154"/>
+    <mergeCell ref="B159:C159"/>
+    <mergeCell ref="B164:C164"/>
+    <mergeCell ref="B185:C185"/>
+    <mergeCell ref="B188:C188"/>
+    <mergeCell ref="B193:C193"/>
+    <mergeCell ref="B198:C198"/>
+    <mergeCell ref="B215:C215"/>
+    <mergeCell ref="B218:C218"/>
+    <mergeCell ref="B223:C223"/>
     <mergeCell ref="B246:C246"/>
     <mergeCell ref="B249:C249"/>
     <mergeCell ref="B14:C14"/>
@@ -11755,49 +11967,15 @@
     <mergeCell ref="B89:C89"/>
     <mergeCell ref="B92:C92"/>
     <mergeCell ref="B97:C97"/>
-    <mergeCell ref="B126:C126"/>
-    <mergeCell ref="B228:C228"/>
-    <mergeCell ref="B151:C151"/>
-    <mergeCell ref="B154:C154"/>
-    <mergeCell ref="B159:C159"/>
-    <mergeCell ref="B164:C164"/>
-    <mergeCell ref="B185:C185"/>
-    <mergeCell ref="B188:C188"/>
-    <mergeCell ref="B193:C193"/>
-    <mergeCell ref="B198:C198"/>
-    <mergeCell ref="B215:C215"/>
-    <mergeCell ref="B218:C218"/>
-    <mergeCell ref="B223:C223"/>
-    <mergeCell ref="B367:C367"/>
-    <mergeCell ref="B372:C372"/>
-    <mergeCell ref="B336:C336"/>
-    <mergeCell ref="B254:C254"/>
-    <mergeCell ref="B259:C259"/>
-    <mergeCell ref="B283:C283"/>
-    <mergeCell ref="B359:C359"/>
-    <mergeCell ref="B291:C291"/>
-    <mergeCell ref="B296:C296"/>
-    <mergeCell ref="B323:C323"/>
-    <mergeCell ref="B326:C326"/>
-    <mergeCell ref="B331:C331"/>
-    <mergeCell ref="B362:C362"/>
-    <mergeCell ref="B286:C286"/>
-    <mergeCell ref="B432:C432"/>
-    <mergeCell ref="B435:C435"/>
-    <mergeCell ref="B440:C440"/>
-    <mergeCell ref="B445:C445"/>
-    <mergeCell ref="B395:C395"/>
-    <mergeCell ref="B398:C398"/>
-    <mergeCell ref="B403:C403"/>
-    <mergeCell ref="B408:C408"/>
-    <mergeCell ref="B510:C510"/>
-    <mergeCell ref="B513:C513"/>
-    <mergeCell ref="B518:C518"/>
-    <mergeCell ref="B523:C523"/>
-    <mergeCell ref="B470:C470"/>
-    <mergeCell ref="B473:C473"/>
-    <mergeCell ref="B478:C478"/>
-    <mergeCell ref="B483:C483"/>
+    <mergeCell ref="B102:C102"/>
+    <mergeCell ref="B118:C118"/>
+    <mergeCell ref="B121:C121"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="H9:I9"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Auto backup 2026-07-02 06:35:02
</commit_message>
<xml_diff>
--- a/SwissTechSaqib/Swiss Tech Files 2025/Profit Reports/profit report.xlsx
+++ b/SwissTechSaqib/Swiss Tech Files 2025/Profit Reports/profit report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="X:\SwissTechSaqib\Swiss Tech Files 2025\Profit Reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5177570A-BA1A-404C-8D58-84200F20C6BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2D95657-5801-4E2E-87E0-ABE7C360A134}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{C511F85B-2D97-4B40-9A5D-0F8673C41C5B}"/>
   </bookViews>
@@ -1869,10 +1869,10 @@
     <xf numFmtId="0" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -8856,6 +8856,11 @@
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="E569:F569"/>
+    <mergeCell ref="H510:I510"/>
+    <mergeCell ref="E391:F391"/>
+    <mergeCell ref="E283:F283"/>
+    <mergeCell ref="E335:F335"/>
     <mergeCell ref="E234:F234"/>
     <mergeCell ref="E508:F508"/>
     <mergeCell ref="E448:F448"/>
@@ -8864,11 +8869,6 @@
     <mergeCell ref="E94:F94"/>
     <mergeCell ref="E140:F140"/>
     <mergeCell ref="E188:F188"/>
-    <mergeCell ref="E569:F569"/>
-    <mergeCell ref="H510:I510"/>
-    <mergeCell ref="E391:F391"/>
-    <mergeCell ref="E283:F283"/>
-    <mergeCell ref="E335:F335"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -8891,24 +8891,24 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B2" s="63" t="s">
+      <c r="B2" s="62" t="s">
         <v>196</v>
       </c>
-      <c r="C2" s="63"/>
-      <c r="H2" s="63" t="s">
+      <c r="C2" s="62"/>
+      <c r="H2" s="62" t="s">
         <v>197</v>
       </c>
-      <c r="I2" s="63"/>
+      <c r="I2" s="62"/>
     </row>
     <row r="4" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B4" s="62" t="s">
+      <c r="B4" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C4" s="62"/>
-      <c r="H4" s="62" t="s">
+      <c r="C4" s="63"/>
+      <c r="H4" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="I4" s="62"/>
+      <c r="I4" s="63"/>
     </row>
     <row r="5" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B5" s="18" t="s">
@@ -8961,14 +8961,14 @@
       <c r="I8" s="20"/>
     </row>
     <row r="9" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B9" s="62" t="s">
+      <c r="B9" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C9" s="62"/>
-      <c r="H9" s="62" t="s">
+      <c r="C9" s="63"/>
+      <c r="H9" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="I9" s="62"/>
+      <c r="I9" s="63"/>
     </row>
     <row r="10" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B10" s="18" t="s">
@@ -9013,14 +9013,14 @@
       <c r="I13" s="20"/>
     </row>
     <row r="14" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B14" s="62" t="s">
+      <c r="B14" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C14" s="62"/>
-      <c r="H14" s="62" t="s">
+      <c r="C14" s="63"/>
+      <c r="H14" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="I14" s="62"/>
+      <c r="I14" s="63"/>
     </row>
     <row r="15" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B15" s="18" t="s">
@@ -9141,10 +9141,10 @@
       </c>
     </row>
     <row r="29" spans="2:9" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B29" s="63" t="s">
+      <c r="B29" s="62" t="s">
         <v>213</v>
       </c>
-      <c r="C29" s="63"/>
+      <c r="C29" s="62"/>
     </row>
     <row r="30" spans="2:9" x14ac:dyDescent="0.25">
       <c r="H30" t="s">
@@ -9152,10 +9152,10 @@
       </c>
     </row>
     <row r="32" spans="2:9" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B32" s="62" t="s">
+      <c r="B32" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C32" s="62"/>
+      <c r="C32" s="63"/>
     </row>
     <row r="33" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B33" s="18" t="s">
@@ -9192,10 +9192,10 @@
       <c r="C36" s="20"/>
     </row>
     <row r="37" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B37" s="62" t="s">
+      <c r="B37" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C37" s="62"/>
+      <c r="C37" s="63"/>
     </row>
     <row r="38" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B38" s="18" t="s">
@@ -9224,10 +9224,10 @@
       <c r="C41" s="20"/>
     </row>
     <row r="42" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B42" s="62" t="s">
+      <c r="B42" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C42" s="62"/>
+      <c r="C42" s="63"/>
     </row>
     <row r="43" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B43" s="18" t="s">
@@ -9302,16 +9302,16 @@
       </c>
     </row>
     <row r="58" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B58" s="63" t="s">
+      <c r="B58" s="62" t="s">
         <v>215</v>
       </c>
-      <c r="C58" s="63"/>
+      <c r="C58" s="62"/>
     </row>
     <row r="61" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B61" s="62" t="s">
+      <c r="B61" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C61" s="62"/>
+      <c r="C61" s="63"/>
     </row>
     <row r="62" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B62" s="18" t="s">
@@ -9343,10 +9343,10 @@
       <c r="C65" s="20"/>
     </row>
     <row r="66" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B66" s="62" t="s">
+      <c r="B66" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C66" s="62"/>
+      <c r="C66" s="63"/>
     </row>
     <row r="67" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B67" s="18" t="s">
@@ -9374,10 +9374,10 @@
       <c r="C70" s="20"/>
     </row>
     <row r="71" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B71" s="62" t="s">
+      <c r="B71" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C71" s="62"/>
+      <c r="C71" s="63"/>
     </row>
     <row r="72" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B72" s="18" t="s">
@@ -9462,16 +9462,16 @@
       </c>
     </row>
     <row r="89" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B89" s="63" t="s">
+      <c r="B89" s="62" t="s">
         <v>218</v>
       </c>
-      <c r="C89" s="63"/>
+      <c r="C89" s="62"/>
     </row>
     <row r="92" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B92" s="62" t="s">
+      <c r="B92" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C92" s="62"/>
+      <c r="C92" s="63"/>
     </row>
     <row r="93" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B93" s="18" t="s">
@@ -9503,10 +9503,10 @@
       <c r="C96" s="20"/>
     </row>
     <row r="97" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B97" s="62" t="s">
+      <c r="B97" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C97" s="62"/>
+      <c r="C97" s="63"/>
     </row>
     <row r="98" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B98" s="18" t="s">
@@ -9534,10 +9534,10 @@
       <c r="C101" s="20"/>
     </row>
     <row r="102" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B102" s="62" t="s">
+      <c r="B102" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C102" s="62"/>
+      <c r="C102" s="63"/>
     </row>
     <row r="103" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B103" s="18" t="s">
@@ -9618,16 +9618,16 @@
       </c>
     </row>
     <row r="118" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B118" s="63" t="s">
+      <c r="B118" s="62" t="s">
         <v>219</v>
       </c>
-      <c r="C118" s="63"/>
+      <c r="C118" s="62"/>
     </row>
     <row r="121" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B121" s="62" t="s">
+      <c r="B121" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C121" s="62"/>
+      <c r="C121" s="63"/>
     </row>
     <row r="122" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B122" s="18" t="s">
@@ -9659,10 +9659,10 @@
       <c r="C125" s="20"/>
     </row>
     <row r="126" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B126" s="62" t="s">
+      <c r="B126" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C126" s="62"/>
+      <c r="C126" s="63"/>
     </row>
     <row r="127" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B127" s="18" t="s">
@@ -9690,10 +9690,10 @@
       <c r="C130" s="20"/>
     </row>
     <row r="131" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B131" s="62" t="s">
+      <c r="B131" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C131" s="62"/>
+      <c r="C131" s="63"/>
     </row>
     <row r="132" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B132" s="18" t="s">
@@ -9778,16 +9778,16 @@
       </c>
     </row>
     <row r="151" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B151" s="63" t="s">
+      <c r="B151" s="62" t="s">
         <v>220</v>
       </c>
-      <c r="C151" s="63"/>
+      <c r="C151" s="62"/>
     </row>
     <row r="154" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B154" s="62" t="s">
+      <c r="B154" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C154" s="62"/>
+      <c r="C154" s="63"/>
     </row>
     <row r="155" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B155" s="18" t="s">
@@ -9819,10 +9819,10 @@
       <c r="C158" s="20"/>
     </row>
     <row r="159" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B159" s="62" t="s">
+      <c r="B159" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C159" s="62"/>
+      <c r="C159" s="63"/>
     </row>
     <row r="160" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B160" s="18" t="s">
@@ -9850,10 +9850,10 @@
       <c r="C163" s="20"/>
     </row>
     <row r="164" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B164" s="62" t="s">
+      <c r="B164" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C164" s="62"/>
+      <c r="C164" s="63"/>
     </row>
     <row r="165" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B165" s="18" t="s">
@@ -9958,16 +9958,16 @@
       </c>
     </row>
     <row r="185" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B185" s="63" t="s">
+      <c r="B185" s="62" t="s">
         <v>224</v>
       </c>
-      <c r="C185" s="63"/>
+      <c r="C185" s="62"/>
     </row>
     <row r="188" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B188" s="62" t="s">
+      <c r="B188" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C188" s="62"/>
+      <c r="C188" s="63"/>
     </row>
     <row r="189" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B189" s="18" t="s">
@@ -9999,10 +9999,10 @@
       <c r="C192" s="20"/>
     </row>
     <row r="193" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B193" s="62" t="s">
+      <c r="B193" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C193" s="62"/>
+      <c r="C193" s="63"/>
     </row>
     <row r="194" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B194" s="18" t="s">
@@ -10030,10 +10030,10 @@
       <c r="C197" s="20"/>
     </row>
     <row r="198" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B198" s="62" t="s">
+      <c r="B198" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C198" s="62"/>
+      <c r="C198" s="63"/>
     </row>
     <row r="199" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B199" s="18" t="s">
@@ -10134,16 +10134,16 @@
       </c>
     </row>
     <row r="215" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B215" s="63" t="s">
+      <c r="B215" s="62" t="s">
         <v>225</v>
       </c>
-      <c r="C215" s="63"/>
+      <c r="C215" s="62"/>
     </row>
     <row r="218" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B218" s="62" t="s">
+      <c r="B218" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C218" s="62"/>
+      <c r="C218" s="63"/>
     </row>
     <row r="219" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B219" s="18" t="s">
@@ -10175,10 +10175,10 @@
       <c r="C222" s="20"/>
     </row>
     <row r="223" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B223" s="62" t="s">
+      <c r="B223" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C223" s="62"/>
+      <c r="C223" s="63"/>
     </row>
     <row r="224" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B224" s="18" t="s">
@@ -10206,10 +10206,10 @@
       <c r="C227" s="20"/>
     </row>
     <row r="228" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B228" s="62" t="s">
+      <c r="B228" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C228" s="62"/>
+      <c r="C228" s="63"/>
     </row>
     <row r="229" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B229" s="18" t="s">
@@ -10316,16 +10316,16 @@
       </c>
     </row>
     <row r="246" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B246" s="63" t="s">
+      <c r="B246" s="62" t="s">
         <v>228</v>
       </c>
-      <c r="C246" s="63"/>
+      <c r="C246" s="62"/>
     </row>
     <row r="249" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B249" s="62" t="s">
+      <c r="B249" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C249" s="62"/>
+      <c r="C249" s="63"/>
     </row>
     <row r="250" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B250" s="18" t="s">
@@ -10357,10 +10357,10 @@
       <c r="C253" s="20"/>
     </row>
     <row r="254" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B254" s="62" t="s">
+      <c r="B254" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C254" s="62"/>
+      <c r="C254" s="63"/>
     </row>
     <row r="255" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B255" s="18" t="s">
@@ -10388,10 +10388,10 @@
       <c r="C258" s="20"/>
     </row>
     <row r="259" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B259" s="62" t="s">
+      <c r="B259" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C259" s="62"/>
+      <c r="C259" s="63"/>
     </row>
     <row r="260" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B260" s="18" t="s">
@@ -10514,16 +10514,16 @@
       </c>
     </row>
     <row r="283" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B283" s="63" t="s">
+      <c r="B283" s="62" t="s">
         <v>231</v>
       </c>
-      <c r="C283" s="63"/>
+      <c r="C283" s="62"/>
     </row>
     <row r="286" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B286" s="62" t="s">
+      <c r="B286" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C286" s="62"/>
+      <c r="C286" s="63"/>
     </row>
     <row r="287" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B287" s="18" t="s">
@@ -10555,10 +10555,10 @@
       <c r="C290" s="20"/>
     </row>
     <row r="291" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B291" s="62" t="s">
+      <c r="B291" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C291" s="62"/>
+      <c r="C291" s="63"/>
     </row>
     <row r="292" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B292" s="18" t="s">
@@ -10586,10 +10586,10 @@
       <c r="C295" s="20"/>
     </row>
     <row r="296" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B296" s="62" t="s">
+      <c r="B296" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C296" s="62"/>
+      <c r="C296" s="63"/>
     </row>
     <row r="297" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B297" s="18" t="s">
@@ -10704,16 +10704,16 @@
       </c>
     </row>
     <row r="323" spans="2:8" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B323" s="63" t="s">
+      <c r="B323" s="62" t="s">
         <v>232</v>
       </c>
-      <c r="C323" s="63"/>
+      <c r="C323" s="62"/>
     </row>
     <row r="326" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B326" s="62" t="s">
+      <c r="B326" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C326" s="62"/>
+      <c r="C326" s="63"/>
     </row>
     <row r="327" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B327" s="18" t="s">
@@ -10748,10 +10748,10 @@
       <c r="C330" s="20"/>
     </row>
     <row r="331" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B331" s="62" t="s">
+      <c r="B331" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C331" s="62"/>
+      <c r="C331" s="63"/>
     </row>
     <row r="332" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B332" s="18" t="s">
@@ -10779,10 +10779,10 @@
       <c r="C335" s="20"/>
     </row>
     <row r="336" spans="2:8" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B336" s="62" t="s">
+      <c r="B336" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C336" s="62"/>
+      <c r="C336" s="63"/>
     </row>
     <row r="337" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B337" s="18" t="s">
@@ -10875,16 +10875,16 @@
       </c>
     </row>
     <row r="359" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B359" s="63" t="s">
+      <c r="B359" s="62" t="s">
         <v>259</v>
       </c>
-      <c r="C359" s="63"/>
+      <c r="C359" s="62"/>
     </row>
     <row r="362" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B362" s="62" t="s">
+      <c r="B362" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C362" s="62"/>
+      <c r="C362" s="63"/>
     </row>
     <row r="363" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B363" s="18" t="s">
@@ -10916,10 +10916,10 @@
       <c r="C366" s="20"/>
     </row>
     <row r="367" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B367" s="62" t="s">
+      <c r="B367" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C367" s="62"/>
+      <c r="C367" s="63"/>
     </row>
     <row r="368" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B368" s="18" t="s">
@@ -10947,10 +10947,10 @@
       <c r="C371" s="20"/>
     </row>
     <row r="372" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B372" s="62" t="s">
+      <c r="B372" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C372" s="62"/>
+      <c r="C372" s="63"/>
     </row>
     <row r="373" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B373" s="18" t="s">
@@ -11047,16 +11047,16 @@
       </c>
     </row>
     <row r="395" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B395" s="63" t="s">
+      <c r="B395" s="62" t="s">
         <v>302</v>
       </c>
-      <c r="C395" s="63"/>
+      <c r="C395" s="62"/>
     </row>
     <row r="398" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B398" s="62" t="s">
+      <c r="B398" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C398" s="62"/>
+      <c r="C398" s="63"/>
     </row>
     <row r="399" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B399" s="18" t="s">
@@ -11088,10 +11088,10 @@
       <c r="C402" s="20"/>
     </row>
     <row r="403" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B403" s="62" t="s">
+      <c r="B403" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C403" s="62"/>
+      <c r="C403" s="63"/>
     </row>
     <row r="404" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B404" s="18" t="s">
@@ -11119,10 +11119,10 @@
       <c r="C407" s="20"/>
     </row>
     <row r="408" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B408" s="62" t="s">
+      <c r="B408" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C408" s="62"/>
+      <c r="C408" s="63"/>
     </row>
     <row r="409" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B409" s="18" t="s">
@@ -11219,16 +11219,16 @@
       </c>
     </row>
     <row r="432" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B432" s="63" t="s">
+      <c r="B432" s="62" t="s">
         <v>314</v>
       </c>
-      <c r="C432" s="63"/>
+      <c r="C432" s="62"/>
     </row>
     <row r="435" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B435" s="62" t="s">
+      <c r="B435" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C435" s="62"/>
+      <c r="C435" s="63"/>
     </row>
     <row r="436" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B436" s="18" t="s">
@@ -11260,10 +11260,10 @@
       <c r="C439" s="20"/>
     </row>
     <row r="440" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B440" s="62" t="s">
+      <c r="B440" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C440" s="62"/>
+      <c r="C440" s="63"/>
     </row>
     <row r="441" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B441" s="18" t="s">
@@ -11291,10 +11291,10 @@
       <c r="C444" s="20"/>
     </row>
     <row r="445" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B445" s="62" t="s">
+      <c r="B445" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C445" s="62"/>
+      <c r="C445" s="63"/>
     </row>
     <row r="446" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B446" s="18" t="s">
@@ -11391,16 +11391,16 @@
       </c>
     </row>
     <row r="470" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B470" s="63" t="s">
+      <c r="B470" s="62" t="s">
         <v>321</v>
       </c>
-      <c r="C470" s="63"/>
+      <c r="C470" s="62"/>
     </row>
     <row r="473" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B473" s="62" t="s">
+      <c r="B473" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C473" s="62"/>
+      <c r="C473" s="63"/>
     </row>
     <row r="474" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B474" s="18" t="s">
@@ -11432,10 +11432,10 @@
       <c r="C477" s="20"/>
     </row>
     <row r="478" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B478" s="62" t="s">
+      <c r="B478" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C478" s="62"/>
+      <c r="C478" s="63"/>
     </row>
     <row r="479" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B479" s="18" t="s">
@@ -11463,10 +11463,10 @@
       <c r="C482" s="20"/>
     </row>
     <row r="483" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B483" s="62" t="s">
+      <c r="B483" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C483" s="62"/>
+      <c r="C483" s="63"/>
     </row>
     <row r="484" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B484" s="18" t="s">
@@ -11563,16 +11563,16 @@
       </c>
     </row>
     <row r="510" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B510" s="63" t="s">
+      <c r="B510" s="62" t="s">
         <v>328</v>
       </c>
-      <c r="C510" s="63"/>
+      <c r="C510" s="62"/>
     </row>
     <row r="513" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B513" s="62" t="s">
+      <c r="B513" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C513" s="62"/>
+      <c r="C513" s="63"/>
     </row>
     <row r="514" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B514" s="18" t="s">
@@ -11604,10 +11604,10 @@
       <c r="C517" s="20"/>
     </row>
     <row r="518" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B518" s="62" t="s">
+      <c r="B518" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C518" s="62"/>
+      <c r="C518" s="63"/>
     </row>
     <row r="519" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B519" s="18" t="s">
@@ -11635,10 +11635,10 @@
       <c r="C522" s="20"/>
     </row>
     <row r="523" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B523" s="62" t="s">
+      <c r="B523" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C523" s="62"/>
+      <c r="C523" s="63"/>
     </row>
     <row r="524" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B524" s="18" t="s">
@@ -11735,16 +11735,16 @@
       </c>
     </row>
     <row r="552" spans="2:3" ht="26.25" x14ac:dyDescent="0.4">
-      <c r="B552" s="63" t="s">
+      <c r="B552" s="62" t="s">
         <v>363</v>
       </c>
-      <c r="C552" s="63"/>
+      <c r="C552" s="62"/>
     </row>
     <row r="555" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B555" s="62" t="s">
+      <c r="B555" s="63" t="s">
         <v>198</v>
       </c>
-      <c r="C555" s="62"/>
+      <c r="C555" s="63"/>
     </row>
     <row r="556" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B556" s="18" t="s">
@@ -11776,10 +11776,10 @@
       <c r="C559" s="20"/>
     </row>
     <row r="560" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B560" s="62" t="s">
+      <c r="B560" s="63" t="s">
         <v>202</v>
       </c>
-      <c r="C560" s="62"/>
+      <c r="C560" s="63"/>
     </row>
     <row r="561" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B561" s="18" t="s">
@@ -11807,10 +11807,10 @@
       <c r="C564" s="20"/>
     </row>
     <row r="565" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
-      <c r="B565" s="62" t="s">
+      <c r="B565" s="63" t="s">
         <v>205</v>
       </c>
-      <c r="C565" s="62"/>
+      <c r="C565" s="63"/>
     </row>
     <row r="566" spans="2:3" ht="18.75" x14ac:dyDescent="0.3">
       <c r="B566" s="18" t="s">
@@ -11904,38 +11904,30 @@
     </row>
   </sheetData>
   <mergeCells count="72">
-    <mergeCell ref="B552:C552"/>
-    <mergeCell ref="B555:C555"/>
-    <mergeCell ref="B560:C560"/>
-    <mergeCell ref="B565:C565"/>
-    <mergeCell ref="B510:C510"/>
-    <mergeCell ref="B513:C513"/>
-    <mergeCell ref="B518:C518"/>
-    <mergeCell ref="B523:C523"/>
-    <mergeCell ref="B470:C470"/>
-    <mergeCell ref="B473:C473"/>
-    <mergeCell ref="B478:C478"/>
-    <mergeCell ref="B483:C483"/>
-    <mergeCell ref="B432:C432"/>
-    <mergeCell ref="B435:C435"/>
-    <mergeCell ref="B440:C440"/>
-    <mergeCell ref="B445:C445"/>
-    <mergeCell ref="B395:C395"/>
-    <mergeCell ref="B398:C398"/>
-    <mergeCell ref="B403:C403"/>
-    <mergeCell ref="B408:C408"/>
-    <mergeCell ref="B367:C367"/>
-    <mergeCell ref="B372:C372"/>
-    <mergeCell ref="B336:C336"/>
-    <mergeCell ref="B254:C254"/>
-    <mergeCell ref="B259:C259"/>
-    <mergeCell ref="B283:C283"/>
-    <mergeCell ref="B359:C359"/>
-    <mergeCell ref="B291:C291"/>
-    <mergeCell ref="B296:C296"/>
-    <mergeCell ref="B323:C323"/>
-    <mergeCell ref="B326:C326"/>
-    <mergeCell ref="B331:C331"/>
+    <mergeCell ref="B118:C118"/>
+    <mergeCell ref="B121:C121"/>
+    <mergeCell ref="B2:C2"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="H4:I4"/>
+    <mergeCell ref="B9:C9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="B249:C249"/>
+    <mergeCell ref="B14:C14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="B29:C29"/>
+    <mergeCell ref="B32:C32"/>
+    <mergeCell ref="B37:C37"/>
+    <mergeCell ref="B42:C42"/>
+    <mergeCell ref="B131:C131"/>
+    <mergeCell ref="B58:C58"/>
+    <mergeCell ref="B61:C61"/>
+    <mergeCell ref="B66:C66"/>
+    <mergeCell ref="B71:C71"/>
+    <mergeCell ref="B89:C89"/>
+    <mergeCell ref="B92:C92"/>
+    <mergeCell ref="B97:C97"/>
+    <mergeCell ref="B102:C102"/>
     <mergeCell ref="B362:C362"/>
     <mergeCell ref="B286:C286"/>
     <mergeCell ref="B126:C126"/>
@@ -11952,30 +11944,38 @@
     <mergeCell ref="B218:C218"/>
     <mergeCell ref="B223:C223"/>
     <mergeCell ref="B246:C246"/>
-    <mergeCell ref="B249:C249"/>
-    <mergeCell ref="B14:C14"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="B29:C29"/>
-    <mergeCell ref="B32:C32"/>
-    <mergeCell ref="B37:C37"/>
-    <mergeCell ref="B42:C42"/>
-    <mergeCell ref="B131:C131"/>
-    <mergeCell ref="B58:C58"/>
-    <mergeCell ref="B61:C61"/>
-    <mergeCell ref="B66:C66"/>
-    <mergeCell ref="B71:C71"/>
-    <mergeCell ref="B89:C89"/>
-    <mergeCell ref="B92:C92"/>
-    <mergeCell ref="B97:C97"/>
-    <mergeCell ref="B102:C102"/>
-    <mergeCell ref="B118:C118"/>
-    <mergeCell ref="B121:C121"/>
-    <mergeCell ref="B2:C2"/>
-    <mergeCell ref="H2:I2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="H4:I4"/>
-    <mergeCell ref="B9:C9"/>
-    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="B336:C336"/>
+    <mergeCell ref="B254:C254"/>
+    <mergeCell ref="B259:C259"/>
+    <mergeCell ref="B283:C283"/>
+    <mergeCell ref="B359:C359"/>
+    <mergeCell ref="B291:C291"/>
+    <mergeCell ref="B296:C296"/>
+    <mergeCell ref="B323:C323"/>
+    <mergeCell ref="B326:C326"/>
+    <mergeCell ref="B331:C331"/>
+    <mergeCell ref="B395:C395"/>
+    <mergeCell ref="B398:C398"/>
+    <mergeCell ref="B403:C403"/>
+    <mergeCell ref="B408:C408"/>
+    <mergeCell ref="B367:C367"/>
+    <mergeCell ref="B372:C372"/>
+    <mergeCell ref="B470:C470"/>
+    <mergeCell ref="B473:C473"/>
+    <mergeCell ref="B478:C478"/>
+    <mergeCell ref="B483:C483"/>
+    <mergeCell ref="B432:C432"/>
+    <mergeCell ref="B435:C435"/>
+    <mergeCell ref="B440:C440"/>
+    <mergeCell ref="B445:C445"/>
+    <mergeCell ref="B552:C552"/>
+    <mergeCell ref="B555:C555"/>
+    <mergeCell ref="B560:C560"/>
+    <mergeCell ref="B565:C565"/>
+    <mergeCell ref="B510:C510"/>
+    <mergeCell ref="B513:C513"/>
+    <mergeCell ref="B518:C518"/>
+    <mergeCell ref="B523:C523"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>